<commit_message>
docs: record the corpus freeze
</commit_message>
<xml_diff>
--- a/docs/agentic-qa-adoption.xlsx
+++ b/docs/agentic-qa-adoption.xlsx
@@ -1519,7 +1519,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>Approvals and the ledger viewer are the human surface a terminal cannot give. Also the demo that sells the idea.</t>
+          <t>Approvals and the ledger viewer are the human surface a terminal cannot give. Also the demo that sells the idea. A 0.1.0 .vsix already exists in extension/ (Sept) — scope what it does before sizing this.</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Partly there</t>
         </is>
       </c>
     </row>

</xml_diff>